<commit_message>
fix: add template produksi, mit, moc
</commit_message>
<xml_diff>
--- a/frontend/public/templates/Template MIT Quartal.xlsx
+++ b/frontend/public/templates/Template MIT Quartal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/farrelarrizal/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS ZENBOOK\Documents\1. College\Project\3. Pertamina\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9755ACC6-F15D-A14A-9DF2-93DF8CF81826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48F8D16-8800-44C4-AA92-E997932BF425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="2000" windowWidth="27640" windowHeight="16940" xr2:uid="{0B7EFD56-CD58-CC40-91CF-4D30E8DE81C2}"/>
+    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="9960" xr2:uid="{0B7EFD56-CD58-CC40-91CF-4D30E8DE81C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
-  <si>
-    <t>Area</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>MIT Declaration Date</t>
   </si>
@@ -87,9 +84,6 @@
   </si>
   <si>
     <t>Closing Date</t>
-  </si>
-  <si>
-    <t>No Registration - Lokasi</t>
   </si>
   <si>
     <t>No Registration - Jenis MIT</t>
@@ -518,31 +512,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F76B2F-11E0-564D-B111-E3C1876BE770}">
-  <dimension ref="A1:Z1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:X1"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.1640625" customWidth="1"/>
-    <col min="3" max="3" width="29.83203125" customWidth="1"/>
-    <col min="4" max="6" width="29.5" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" customWidth="1"/>
-    <col min="8" max="8" width="17.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.33203125" customWidth="1"/>
-    <col min="10" max="10" width="21" customWidth="1"/>
-    <col min="11" max="11" width="18.6640625" customWidth="1"/>
-    <col min="12" max="12" width="33.1640625" customWidth="1"/>
-    <col min="13" max="13" width="28" customWidth="1"/>
-    <col min="14" max="14" width="26.33203125" customWidth="1"/>
-    <col min="15" max="15" width="21.6640625" customWidth="1"/>
-    <col min="17" max="17" width="29.83203125" customWidth="1"/>
-    <col min="21" max="22" width="34.83203125" customWidth="1"/>
-    <col min="24" max="24" width="18.6640625" customWidth="1"/>
-    <col min="26" max="26" width="20.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.796875" customWidth="1"/>
+    <col min="2" max="4" width="29.5" customWidth="1"/>
+    <col min="5" max="5" width="24.296875" customWidth="1"/>
+    <col min="6" max="6" width="17.796875" customWidth="1"/>
+    <col min="7" max="7" width="18.296875" customWidth="1"/>
+    <col min="8" max="8" width="21" customWidth="1"/>
+    <col min="9" max="9" width="18.69921875" customWidth="1"/>
+    <col min="10" max="10" width="33.19921875" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="26.296875" customWidth="1"/>
+    <col min="13" max="13" width="21.69921875" customWidth="1"/>
+    <col min="15" max="15" width="29.796875" customWidth="1"/>
+    <col min="19" max="20" width="34.796875" customWidth="1"/>
+    <col min="22" max="22" width="18.69921875" customWidth="1"/>
+    <col min="24" max="24" width="20.296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>16</v>
@@ -554,70 +546,64 @@
         <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="V1" s="1" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>